<commit_message>
Move to the InterviewProgram
</commit_message>
<xml_diff>
--- a/TestData.xlsx
+++ b/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Automation Projects\1ARTinterview\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A641C457-86D3-434B-8735-377D49B4E744}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7E2B937-0624-40A6-9DB3-F88AEE6BC0E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11829" xr2:uid="{B2D2FB60-FC6E-4C94-BA16-C29BA5305111}"/>
   </bookViews>
@@ -42,13 +42,13 @@
     <t>Password</t>
   </si>
   <si>
-    <t>pintumagic@gmail.com</t>
+    <t>kpintu123@yopmail.com</t>
   </si>
   <si>
-    <t>pintu!1A</t>
+    <t>asdf</t>
   </si>
   <si>
-    <t>kpintu123@yopmail.com</t>
+    <t>f</t>
   </si>
 </sst>
 </file>
@@ -416,15 +416,15 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B3">
         <v>12345</v>

</xml_diff>